<commit_message>
Actualizacion de RTM y Checklist Turnos/login agregados.
</commit_message>
<xml_diff>
--- a/04-RTM/RTM_cases.xlsx
+++ b/04-RTM/RTM_cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Desktop\Trabajos Personal\Excel de trabajos personales\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Desktop\Trabajos Personal\QA-testing-gestion-turnos-medicos\04-RTM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C6BF3D1-830E-4792-A35E-6650CBDF91FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBB1DFA-57A4-4AF8-A11E-A3CA95E8E919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{36282FB5-5FA0-41D8-9EFF-4106B5102D26}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
   <si>
     <t>Proyecto</t>
   </si>
@@ -84,9 +84,6 @@
     <t>RF-001</t>
   </si>
   <si>
-    <t>RF-002</t>
-  </si>
-  <si>
     <t>RF-008</t>
   </si>
   <si>
@@ -114,36 +111,18 @@
     <t>Gestión de Pacientes</t>
   </si>
   <si>
-    <t>TC-PAC-001 al TC-PAC-006, TC-PAC-012, TC-PAC-014, TC-PAC-015</t>
-  </si>
-  <si>
-    <t>Cubierto</t>
-  </si>
-  <si>
     <t>Validación de Pacientes</t>
   </si>
   <si>
-    <t>TC-PAC-007 al TC-PAC-011, TC-PAC-013</t>
-  </si>
-  <si>
     <t>Reserva de Turnos</t>
   </si>
   <si>
-    <t>TC-TUR-001, TC-TUR-003, TC-TUR-015</t>
-  </si>
-  <si>
     <t>Validación de Disponibilidad</t>
   </si>
   <si>
-    <t>TC-TUR-004, TC-TUR-007, TC-TUR-008, TC-TUR-009</t>
-  </si>
-  <si>
     <t>Control de Superposición</t>
   </si>
   <si>
-    <t>TC-TUR-005, TC-TUR-010</t>
-  </si>
-  <si>
     <t>Búsqueda de Turnos</t>
   </si>
   <si>
@@ -165,20 +144,65 @@
     <t>Cancelación de Turnos</t>
   </si>
   <si>
-    <t>TC-TUR-013, TC-TUR-014</t>
-  </si>
-  <si>
     <t>Autenticación</t>
   </si>
   <si>
-    <t>TC-LOGIN-001 al TC-LOGIN-015</t>
+    <t xml:space="preserve">RF-002 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-TUR-004, TC-TUR-007, TC-TUR-008, TC-TUR-009 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-TUR-005, TC-TUR-010 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-TUR-001, TC-TUR-003, TC-TUR-015 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-TUR-013, TC-TUR-014 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-LOGIN-001 al TC-LOGIN-015 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-PAC-007 al TC-PAC-011, TC-PAC-013 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-PAC-001 al TC-PAC-006, TC-PAC-012, TC-PAC-014, TC-PAC-015 </t>
+  </si>
+  <si>
+    <t>Módulo</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Pacientes</t>
+  </si>
+  <si>
+    <t>Turnos</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> RF-016  </t>
+  </si>
+  <si>
+    <t>Gestión de Permisos</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>No incluido.</t>
+  </si>
+  <si>
+    <t>Cubierto.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -204,6 +228,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -235,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -258,6 +290,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -572,14 +605,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9CFA65B-3CBB-46A4-AAD6-B2B83A80508E}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" customWidth="1"/>
     <col min="3" max="3" width="39.140625" customWidth="1"/>
+    <col min="4" max="4" width="47.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -588,7 +622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
@@ -596,13 +630,13 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="3"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
@@ -610,7 +644,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
@@ -618,7 +652,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
@@ -626,158 +660,209 @@
         <v>46234</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D12" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="6" t="s">
+      <c r="D14" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="E16" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="6" t="s">
+      <c r="D17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="E17" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="6" t="s">
+      <c r="D18" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="E18" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="6" t="s">
+      <c r="D19" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H19" s="8"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="6" t="s">
+      <c r="D20" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>26</v>
+      <c r="E20" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>